<commit_message>
fix(archery): retune sway data for hand-tremor shape (both maps)
shake_free_seconds 0.8→0.0 (no more free window — fatigue starts
counting immediately), shake_ramp_seconds 1.5→2.5 (fatigue builds over
the whole hold now that it starts at 0), shake_max_degrees 0.4→0.25
(the 22° drawn zoom magnifies the same angle ~2.7x vs. the 60° undrawn
FOV). Applies to both archery rows (map 5 and map 6).

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01J3Xe7rZoLKi3dJFGKrLsGL
</commit_message>
<xml_diff>
--- a/table/Datas/#ArcheryConfig.xlsx
+++ b/table/Datas/#ArcheryConfig.xlsx
@@ -791,13 +791,13 @@
         <v>1</v>
       </c>
       <c r="L5" t="n">
-        <v>0.8</v>
+        <v>0</v>
       </c>
       <c r="M5" t="n">
-        <v>1.5</v>
+        <v>2.5</v>
       </c>
       <c r="N5" t="n">
-        <v>0.4</v>
+        <v>0.25</v>
       </c>
       <c r="O5" t="n">
         <v>1.2</v>
@@ -856,13 +856,13 @@
         <v>1</v>
       </c>
       <c r="L6" t="n">
-        <v>0.8</v>
+        <v>0</v>
       </c>
       <c r="M6" t="n">
-        <v>1.5</v>
+        <v>2.5</v>
       </c>
       <c r="N6" t="n">
-        <v>0.4</v>
+        <v>0.25</v>
       </c>
       <c r="O6" t="n">
         <v>1.2</v>

</xml_diff>

<commit_message>
fix(archery): add shake_base_ratio column (0.4, both maps)
New column appended at the far right (Luban reads by position) since the
sway shape needed a baseline-tremor term the ramp-from-zero fatigue curve
couldn't provide — see the LOP-Shared ArcheryShake.Offset fix in the same
slice. 0.4 means a bow trembles at ~40% of shake_max_degrees the instant
it's held, rising to 100% only once fatigue (shake_ramp_seconds) fully
kicks in.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01J3Xe7rZoLKi3dJFGKrLsGL
</commit_message>
<xml_diff>
--- a/table/Datas/#ArcheryConfig.xlsx
+++ b/table/Datas/#ArcheryConfig.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V6"/>
+  <dimension ref="A1:W6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -527,6 +527,11 @@
           <t>match_duration_ticks</t>
         </is>
       </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>shake_base_ratio</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -639,6 +644,11 @@
           <t>int</t>
         </is>
       </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -756,6 +766,11 @@
       <c r="V4" t="inlineStr">
         <is>
           <t>match_duration_ticks</t>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>shake_base_ratio</t>
         </is>
       </c>
     </row>
@@ -823,6 +838,9 @@
       <c r="V5" t="n">
         <v>3000</v>
       </c>
+      <c r="W5" t="n">
+        <v>0.4</v>
+      </c>
     </row>
     <row r="6">
       <c r="B6" t="n">
@@ -887,6 +905,9 @@
       </c>
       <c r="V6" t="n">
         <v>0</v>
+      </c>
+      <c r="W6" t="n">
+        <v>0.4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>